<commit_message>
feat: add shotgun pellet spread
</commit_message>
<xml_diff>
--- a/Config/Excel/DT_WeaponFireModeConfig.xlsx
+++ b/Config/Excel/DT_WeaponFireModeConfig.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workspace\letsdeeprock-profession-preview\com-final-serial\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workspace\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{194F830D-52DC-4FEF-BF20-7051738B2488}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F88439EE-41A9-4253-8F9B-57630AFEFFD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1087,7 +1087,7 @@
         <v>1</v>
       </c>
       <c r="U6">
-        <v>12</v>
+        <v>60</v>
       </c>
       <c r="V6">
         <v>1</v>

</xml_diff>

<commit_message>
feat: add weapon falloff and recoil
</commit_message>
<xml_diff>
--- a/Config/Excel/DT_WeaponFireModeConfig.xlsx
+++ b/Config/Excel/DT_WeaponFireModeConfig.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workspace\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\testfiles\UnrealDeepRock\LetsDeepRock\Config\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F88439EE-41A9-4253-8F9B-57630AFEFFD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E22F0353-FA02-4E28-8A18-F986B7BD79A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="103">
   <si>
     <t>#TABLE=DT_WeaponFireModeConfig</t>
   </si>
@@ -127,6 +127,15 @@
     <t>DamageFalloffEnd</t>
   </si>
   <si>
+    <t>StatusEffectId</t>
+  </si>
+  <si>
+    <t>ProjectileGravityScale</t>
+  </si>
+  <si>
+    <t>MaxHitTargets</t>
+  </si>
+  <si>
     <t>射击模式ID</t>
   </si>
   <si>
@@ -196,124 +205,99 @@
     <t>衰减终点</t>
   </si>
   <si>
+    <t>异常状态ID</t>
+  </si>
+  <si>
+    <t>投射物重力倍率</t>
+  </si>
+  <si>
+    <t>最大命中目标数</t>
+  </si>
+  <si>
+    <t>Ranger_ArcaneCrossbow_RapidBolt</t>
+  </si>
+  <si>
+    <t>游侠奥术连弩高速弩箭</t>
+  </si>
+  <si>
+    <t>高速弩箭</t>
+  </si>
+  <si>
     <t>Hold</t>
   </si>
   <si>
     <t>Damage.Type.Physical</t>
   </si>
   <si>
+    <t>Vulnerable</t>
+  </si>
+  <si>
+    <t>Ranger_SawedOffShotgun_Default</t>
+  </si>
+  <si>
+    <t>近距离八弹丸爆发</t>
+  </si>
+  <si>
+    <t>短管霰弹</t>
+  </si>
+  <si>
+    <t>Press</t>
+  </si>
+  <si>
+    <t>Ranger_FullAutoPistol_Default</t>
+  </si>
+  <si>
+    <t>全距离稳定连射</t>
+  </si>
+  <si>
+    <t>全自动手枪</t>
+  </si>
+  <si>
+    <t>Ranger_ThrowingKnife_Default</t>
+  </si>
+  <si>
+    <t>高单体抛物线投射</t>
+  </si>
+  <si>
+    <t>飞刀</t>
+  </si>
+  <si>
+    <t>Demolitionist_Flamethrower_Default</t>
+  </si>
+  <si>
+    <t>近距离持续火焰伤害</t>
+  </si>
+  <si>
+    <t>火焰喷射</t>
+  </si>
+  <si>
+    <t>Damage.Type.Fire</t>
+  </si>
+  <si>
+    <t>Burning</t>
+  </si>
+  <si>
+    <t>Demolitionist_Revolver_Default</t>
+  </si>
+  <si>
+    <t>高伤害高精度单发</t>
+  </si>
+  <si>
+    <t>左轮射击</t>
+  </si>
+  <si>
+    <t>Demolitionist_RocketLauncher_Default</t>
+  </si>
+  <si>
+    <t>低频范围爆炸</t>
+  </si>
+  <si>
+    <t>火箭射击</t>
+  </si>
+  <si>
     <t>Damage.Type.Explosion</t>
   </si>
   <si>
-    <t>StatusEffectId</t>
-  </si>
-  <si>
-    <t>ProjectileGravityScale</t>
-  </si>
-  <si>
-    <t>MaxHitTargets</t>
-  </si>
-  <si>
-    <t>异常状态ID</t>
-  </si>
-  <si>
-    <t>投射物重力倍率</t>
-  </si>
-  <si>
-    <t>最大命中目标数</t>
-  </si>
-  <si>
-    <t>Ranger_ArcaneCrossbow_RapidBolt</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>游侠奥术连弩高速弩箭</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>高速弩箭</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Hold</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Damage.Type.Physical</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Vulnerable</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Ranger_SawedOffShotgun_Default</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>近距离八弹丸爆发</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>短管霰弹</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Press</t>
-  </si>
-  <si>
-    <t>Press</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Ranger_FullAutoPistol_Default</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>全距离稳定连射</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>全自动手枪</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Ranger_ThrowingKnife_Default</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>高单体抛物线投射</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>飞刀</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>近距离持续火焰伤害</t>
-  </si>
-  <si>
-    <t>火焰喷射</t>
-  </si>
-  <si>
-    <t>Damage.Type.Fire</t>
-  </si>
-  <si>
-    <t>Burning</t>
-  </si>
-  <si>
-    <t>高伤害高精度单发</t>
-  </si>
-  <si>
-    <t>左轮射击</t>
-  </si>
-  <si>
-    <t>低频范围爆炸</t>
-  </si>
-  <si>
-    <t>火箭射击</t>
-  </si>
-  <si>
     <t>Engineer_AssaultRifle_Default</t>
   </si>
   <si>
@@ -335,16 +319,16 @@
     <t>Bleeding</t>
   </si>
   <si>
-    <t>Demolitionist_Flamethrower_Default</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Demolitionist_Revolver_Default</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Demolitionist_RocketLauncher_Default</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+    <t>Ranger_ArcaneCrossbow_ChargedArcaneMissile</t>
+  </si>
+  <si>
+    <t>游侠奥术连弩蓄力范围飞弹</t>
+  </si>
+  <si>
+    <t>蓄力奥术飞弹</t>
+  </si>
+  <si>
+    <t>Charge</t>
   </si>
 </sst>
 </file>
@@ -691,7 +675,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AA13"/>
+  <dimension ref="A1:AA14"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <sheetData>
     <row r="1" spans="1:27" x14ac:dyDescent="0.15">
@@ -862,113 +846,113 @@
         <v>34</v>
       </c>
       <c r="Y3" t="s">
-        <v>61</v>
+        <v>35</v>
       </c>
       <c r="Z3" t="s">
-        <v>62</v>
+        <v>36</v>
       </c>
       <c r="AA3" t="s">
-        <v>63</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.15">
       <c r="A4" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B4" t="s">
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D4" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E4" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F4" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="G4" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="H4" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="I4" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="J4" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="K4" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="L4" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="M4" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="N4" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="O4" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="P4" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="Q4" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="R4" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="S4" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="T4" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="U4" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="V4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="W4" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="X4" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="Y4" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="Z4" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="AA4" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.15">
       <c r="A5" t="s">
+        <v>64</v>
+      </c>
+      <c r="B5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C5" t="s">
+        <v>66</v>
+      </c>
+      <c r="D5" t="s">
         <v>67</v>
       </c>
-      <c r="B5" t="s">
+      <c r="G5" t="s">
         <v>68</v>
-      </c>
-      <c r="C5" t="s">
-        <v>69</v>
-      </c>
-      <c r="D5" t="s">
-        <v>70</v>
-      </c>
-      <c r="G5" t="s">
-        <v>71</v>
       </c>
       <c r="H5">
         <v>12</v>
@@ -1022,7 +1006,7 @@
         <v>0</v>
       </c>
       <c r="Y5" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="Z5">
         <v>0</v>
@@ -1033,19 +1017,19 @@
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.15">
       <c r="A6" t="s">
+        <v>70</v>
+      </c>
+      <c r="B6" t="s">
+        <v>71</v>
+      </c>
+      <c r="C6" t="s">
+        <v>72</v>
+      </c>
+      <c r="D6" t="s">
         <v>73</v>
       </c>
-      <c r="B6" t="s">
-        <v>74</v>
-      </c>
-      <c r="C6" t="s">
-        <v>75</v>
-      </c>
-      <c r="D6" t="s">
-        <v>77</v>
-      </c>
       <c r="G6" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="H6">
         <v>8</v>
@@ -1107,19 +1091,19 @@
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.15">
       <c r="A7" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B7" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="C7" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="D7" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="G7" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="H7">
         <v>14</v>
@@ -1167,10 +1151,10 @@
         <v>0.25</v>
       </c>
       <c r="W7">
-        <v>1200</v>
+        <v>600</v>
       </c>
       <c r="X7">
-        <v>3200</v>
+        <v>1600</v>
       </c>
       <c r="Z7">
         <v>0</v>
@@ -1181,19 +1165,19 @@
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.15">
       <c r="A8" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="B8" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C8" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="D8" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="G8" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="H8">
         <v>55</v>
@@ -1255,19 +1239,19 @@
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.15">
       <c r="A9" t="s">
-        <v>99</v>
+        <v>80</v>
       </c>
       <c r="B9" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C9" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="D9" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="G9" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="H9">
         <v>4</v>
@@ -1321,7 +1305,7 @@
         <v>700</v>
       </c>
       <c r="Y9" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="Z9">
         <v>0</v>
@@ -1332,19 +1316,19 @@
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.15">
       <c r="A10" t="s">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="B10" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C10" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D10" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="G10" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="H10">
         <v>60</v>
@@ -1392,10 +1376,10 @@
         <v>0.8</v>
       </c>
       <c r="W10">
-        <v>1800</v>
+        <v>900</v>
       </c>
       <c r="X10">
-        <v>5000</v>
+        <v>2500</v>
       </c>
       <c r="Z10">
         <v>0</v>
@@ -1406,19 +1390,19 @@
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.15">
       <c r="A11" t="s">
-        <v>101</v>
+        <v>88</v>
       </c>
       <c r="B11" t="s">
+        <v>89</v>
+      </c>
+      <c r="C11" t="s">
         <v>90</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
+        <v>73</v>
+      </c>
+      <c r="G11" t="s">
         <v>91</v>
-      </c>
-      <c r="D11" t="s">
-        <v>76</v>
-      </c>
-      <c r="G11" t="s">
-        <v>60</v>
       </c>
       <c r="H11">
         <v>40</v>
@@ -1489,10 +1473,10 @@
         <v>94</v>
       </c>
       <c r="D12" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="G12" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="H12">
         <v>18</v>
@@ -1563,10 +1547,10 @@
         <v>97</v>
       </c>
       <c r="D13" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="G13" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="H13">
         <v>35</v>
@@ -1627,6 +1611,80 @@
       </c>
       <c r="AA13">
         <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:27" x14ac:dyDescent="0.15">
+      <c r="A14" t="s">
+        <v>99</v>
+      </c>
+      <c r="B14" t="s">
+        <v>100</v>
+      </c>
+      <c r="C14" t="s">
+        <v>101</v>
+      </c>
+      <c r="D14" t="s">
+        <v>102</v>
+      </c>
+      <c r="G14" t="s">
+        <v>91</v>
+      </c>
+      <c r="H14">
+        <v>20</v>
+      </c>
+      <c r="I14">
+        <v>0.05</v>
+      </c>
+      <c r="J14">
+        <v>1</v>
+      </c>
+      <c r="K14">
+        <v>0.8</v>
+      </c>
+      <c r="L14">
+        <v>1.2</v>
+      </c>
+      <c r="M14">
+        <v>2200</v>
+      </c>
+      <c r="N14">
+        <v>4</v>
+      </c>
+      <c r="O14">
+        <v>1</v>
+      </c>
+      <c r="P14">
+        <v>35</v>
+      </c>
+      <c r="Q14">
+        <v>250</v>
+      </c>
+      <c r="R14">
+        <v>0.5</v>
+      </c>
+      <c r="S14">
+        <v>1</v>
+      </c>
+      <c r="T14" t="b">
+        <v>1</v>
+      </c>
+      <c r="U14">
+        <v>0</v>
+      </c>
+      <c r="V14">
+        <v>0</v>
+      </c>
+      <c r="W14">
+        <v>0</v>
+      </c>
+      <c r="X14">
+        <v>0</v>
+      </c>
+      <c r="Z14">
+        <v>0</v>
+      </c>
+      <c r="AA14">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>